<commit_message>
chore: atualiza artefatos de saída do agente (30 relatórios reprocessados)
Resultados da execução após correção dos falsos-positivos E4/E5.
Inclui JSON, pareceres .md, minutas .txt e consolidado .xlsx.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/consolidado_auditoria.xlsx
+++ b/output/consolidado_auditoria.xlsx
@@ -451,15 +451,15 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DEVOLVER PARA REELABORAÇÃO</t>
+          <t>DEVOLVER PARA AJUSTES</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Atividades Realizadas) | E5: Inconsistência no somatório da carga horária. | E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
+          <t>E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
         </is>
       </c>
     </row>
@@ -511,15 +511,15 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DEVOLVER PARA REELABORAÇÃO</t>
+          <t>DEVOLVER PARA AJUSTES</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Atividades Realizadas) | E5: Inconsistência no somatório da carga horária. | E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
+          <t>E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
         </is>
       </c>
     </row>
@@ -591,15 +591,15 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DEVOLVER PARA REELABORAÇÃO</t>
+          <t>DEVOLVER PARA AJUSTES</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Atividades Realizadas) | E5: Inconsistência no somatório da carga horária. | E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
+          <t>E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
         </is>
       </c>
     </row>
@@ -651,15 +651,15 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DEVOLVER PARA REELABORAÇÃO</t>
+          <t>DEVOLVER PARA AJUSTES</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Atividades Realizadas) | E5: Inconsistência no somatório da carga horária. | E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
+          <t>E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
         </is>
       </c>
     </row>
@@ -675,11 +675,11 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Atividades Realizadas, Síntese da Execução) | E5: Inconsistência no somatório da carga horária.</t>
+          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Síntese da Execução)</t>
         </is>
       </c>
     </row>
@@ -711,15 +711,15 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DEVOLVER PARA REELABORAÇÃO</t>
+          <t>DEVOLVER PARA AJUSTES</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Atividades Realizadas) | E5: Inconsistência no somatório da carga horária. | E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
+          <t>E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
         </is>
       </c>
     </row>
@@ -731,15 +731,15 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DEVOLVER PARA AJUSTES</t>
+          <t>DEVOLVER PARA REELABORAÇÃO</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>E2: Bolsista 'César Monteiro' declarado não consta no Edital Oficial para o projeto submetido.</t>
+          <t>Nenhuma</t>
         </is>
       </c>
     </row>
@@ -751,15 +751,15 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DEVOLVER PARA REELABORAÇÃO</t>
+          <t>DEVOLVER PARA AJUSTES</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Atividades Realizadas) | E5: Inconsistência no somatório da carga horária. | E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
+          <t>E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
         </is>
       </c>
     </row>
@@ -771,15 +771,15 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DEVOLVER PARA REELABORAÇÃO</t>
+          <t>DEVOLVER PARA AJUSTES</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Atividades Realizadas) | E5: Inconsistência no somatório da carga horária. | E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
+          <t>E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
         </is>
       </c>
     </row>
@@ -811,15 +811,15 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DEVOLVER PARA REELABORAÇÃO</t>
+          <t>APROVAR</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Atividades Realizadas) | E5: Inconsistência no somatório da carga horária.</t>
+          <t>Nenhuma</t>
         </is>
       </c>
     </row>
@@ -831,15 +831,15 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DEVOLVER PARA REELABORAÇÃO</t>
+          <t>APROVAR</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Atividades Realizadas) | E5: Inconsistência no somatório da carga horária.</t>
+          <t>Nenhuma</t>
         </is>
       </c>
     </row>
@@ -871,15 +871,15 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DEVOLVER PARA REELABORAÇÃO</t>
+          <t>DEVOLVER PARA AJUSTES</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Atividades Realizadas) | E5: Inconsistência no somatório da carga horária. | E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
+          <t>E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
         </is>
       </c>
     </row>
@@ -891,15 +891,15 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DEVOLVER PARA REELABORAÇÃO</t>
+          <t>DEVOLVER PARA AJUSTES</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Atividades Realizadas) | E5: Inconsistência no somatório da carga horária. | E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
+          <t>E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
         </is>
       </c>
     </row>
@@ -931,15 +931,15 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DEVOLVER PARA REELABORAÇÃO</t>
+          <t>APROVAR</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Atividades Realizadas) | E5: Inconsistência no somatório da carga horária.</t>
+          <t>Nenhuma</t>
         </is>
       </c>
     </row>
@@ -975,11 +975,11 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Atividades Realizadas, Resultados Alcançados / Produtos) | E5: Inconsistência no somatório da carga horária. | E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
+          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Resultados Alcançados / Produtos) | E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
         </is>
       </c>
     </row>
@@ -1011,15 +1011,15 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DEVOLVER PARA REELABORAÇÃO</t>
+          <t>DEVOLVER PARA AJUSTES</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>E4: Ausência de campos ou seções obrigatórias no relatório. (Atividades Realizadas) | E5: Inconsistência no somatório da carga horária. | E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
+          <t>E1: Relatório omitiu recursos, mas a base oficial indica que houve fomento.</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1110,11 +1110,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>26.7%</t>
         </is>
       </c>
     </row>
@@ -1125,11 +1125,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>26.7%</t>
+          <t>56.7%</t>
         </is>
       </c>
     </row>
@@ -1140,11 +1140,11 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>56.7%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1180,105 +1180,90 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Erro tipo: E4</t>
+          <t>Erro tipo: E1</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>32.1%</t>
+          <t>45.8%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Erro tipo: E5</t>
+          <t>Erro tipo: Erro na Prestação de Contas</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>28.3%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Erro tipo: E1</t>
+          <t>Erro tipo: Erro E1</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>20.8%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Erro tipo: Erro na Prestação de Contas</t>
+          <t>Erro tipo: E4</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.8%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Erro tipo: Erro E1</t>
+          <t>Erro tipo: E2</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Erro tipo: E2</t>
+          <t>Erro tipo: E3</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>5.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Erro tipo: E3</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1.9%</t>
+          <t>4.2%</t>
         </is>
       </c>
     </row>

</xml_diff>